<commit_message>
upadted BOM and PCB files
</commit_message>
<xml_diff>
--- a/BOM/MechanicalBOM.xlsx
+++ b/BOM/MechanicalBOM.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\模型\谐波赤道仪\GitHub\DIY-Harmonic-Equatorial-Mount\BOM\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D2B963D-A8AC-465D-86A0-7B30C24DDC60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -18,14 +24,116 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="30">
+  <si>
+    <t>名称</t>
+  </si>
+  <si>
+    <t>规格</t>
+  </si>
+  <si>
+    <t>数量</t>
+  </si>
+  <si>
+    <t>塞打螺栓</t>
+  </si>
+  <si>
+    <t>8*10*M6</t>
+  </si>
+  <si>
+    <t>8*8*M6</t>
+  </si>
+  <si>
+    <t>一字塞打螺栓</t>
+  </si>
+  <si>
+    <t>12.9级杯头螺丝</t>
+  </si>
+  <si>
+    <t>M5*18</t>
+  </si>
+  <si>
+    <t>304不锈钢内螺纹圆柱销</t>
+  </si>
+  <si>
+    <t>Φ12*25*M6</t>
+  </si>
+  <si>
+    <t>小微型推力球平面轴承</t>
+  </si>
+  <si>
+    <t>F8-14M 尺寸8*14*4</t>
+  </si>
+  <si>
+    <t>304不锈钢一字塞打螺丝</t>
+  </si>
+  <si>
+    <t>M8*4*M6</t>
+  </si>
+  <si>
+    <t>圆切边法兰铜合金无油衬套黄铜铜套</t>
+  </si>
+  <si>
+    <t>8-15(27*4/8*12*15)-圆光</t>
+  </si>
+  <si>
+    <t>M5*14</t>
+  </si>
+  <si>
+    <t>薄头内六角螺丝钉DIN7984</t>
+  </si>
+  <si>
+    <t>M3*4</t>
+  </si>
+  <si>
+    <t>铜垫片</t>
+  </si>
+  <si>
+    <t>M8*12*0.5</t>
+  </si>
+  <si>
+    <t>M5*9*0.5</t>
+  </si>
+  <si>
+    <t>不锈钢超薄垫片</t>
+  </si>
+  <si>
+    <t>8*12*0.2</t>
+  </si>
+  <si>
+    <t>12.9级薄头内六角螺丝DIN7984</t>
+  </si>
+  <si>
+    <t>M4*16</t>
+  </si>
+  <si>
+    <t>M4*12</t>
+  </si>
+  <si>
+    <t>12.9级高强度镀镍薄头内六角螺丝</t>
+  </si>
+  <si>
+    <t>M6*12</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="1" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -49,11 +157,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -330,10 +441,204 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="32" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.58203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C4" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C10" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C13" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="1">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C17" s="1">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>